<commit_message>
Pre Market Tue 2026-07-07
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-07-07.xlsx
+++ b/market-prep/Pre Market 2026-07-07.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7542,99</t>
+          <t>7537,43</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29794,54</t>
+          <t>29697,87</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>53017,47</t>
+          <t>53055,91</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4163,76</t>
+          <t>4164,53</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>62,07</t>
+          <t>62,04</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1635,90</t>
+          <t>1631,10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>72,14</t>
+          <t>71,99</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>63654,41</t>
+          <t>64171,00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1791,45</t>
+          <t>1813,10</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-3,41%</t>
+          <t>-3,59%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7547,90</t>
+          <t>7537,43</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -768,7 +768,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>44</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>

</xml_diff>